<commit_message>
#24 Custom Supplier Quotes Updated.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/ARC_1.0.5/Client_BOM_ARC_1.0.5.xlsx
+++ b/Deliverables/BOM/ARC_1.0.5/Client_BOM_ARC_1.0.5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Oliver-ARC\Deliverables\BOM\ARC_1.0.5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AEFA288-D115-407A-867E-3F90D182F1AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74CA7600-0C6F-4C60-8889-5BEAF45F7C1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="382">
   <si>
     <t>Component list</t>
   </si>
@@ -1170,13 +1170,13 @@
     <t>Single Board Cost</t>
   </si>
   <si>
-    <t>Need Custom Supplier Quotation</t>
-  </si>
-  <si>
     <t>Bill of Materials for Project [ARC_1.0.5]</t>
   </si>
   <si>
     <t>[ARC_1.0.5]</t>
+  </si>
+  <si>
+    <t>Quantity (5 Boards)</t>
   </si>
 </sst>
 </file>
@@ -1664,7 +1664,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1885,6 +1885,9 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1912,13 +1915,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>10417</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>1724025</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>161925</xdr:rowOff>
@@ -2226,7 +2229,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:X88"/>
+  <dimension ref="A1:Y88"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="26" customWidth="1"/>
@@ -2239,15 +2242,16 @@
     <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="18.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -2263,9 +2267,10 @@
       <c r="M1" s="70"/>
       <c r="N1" s="70"/>
       <c r="O1" s="70"/>
-      <c r="P1" s="71"/>
-    </row>
-    <row r="2" spans="1:24" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P1" s="70"/>
+      <c r="Q1" s="71"/>
+    </row>
+    <row r="2" spans="1:25" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="21"/>
       <c r="C2" s="39"/>
@@ -2274,7 +2279,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="55" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -2285,9 +2290,10 @@
       <c r="M2" s="4"/>
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
-      <c r="P2" s="3"/>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="P2" s="4"/>
+      <c r="Q2" s="3"/>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="22"/>
       <c r="C3" s="40"/>
@@ -2296,7 +2302,7 @@
       </c>
       <c r="E3" s="13"/>
       <c r="F3" s="56" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="5"/>
@@ -2307,9 +2313,10 @@
       <c r="M3" s="5"/>
       <c r="N3" s="5"/>
       <c r="O3" s="5"/>
-      <c r="P3" s="72"/>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="P3" s="5"/>
+      <c r="Q3" s="72"/>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="22"/>
       <c r="C4" s="40"/>
@@ -2318,7 +2325,7 @@
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="57" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="7"/>
@@ -2329,9 +2336,10 @@
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
       <c r="O4" s="6"/>
-      <c r="P4" s="73"/>
-    </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="P4" s="6"/>
+      <c r="Q4" s="73"/>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="22"/>
       <c r="C5" s="40"/>
@@ -2351,9 +2359,10 @@
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
       <c r="O5" s="6"/>
-      <c r="P5" s="73"/>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="P5" s="6"/>
+      <c r="Q5" s="73"/>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="23"/>
       <c r="C6" s="41"/>
@@ -2369,9 +2378,10 @@
       <c r="M6" s="6"/>
       <c r="N6" s="6"/>
       <c r="O6" s="6"/>
-      <c r="P6" s="73"/>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="P6" s="6"/>
+      <c r="Q6" s="73"/>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="24"/>
       <c r="C7" s="42"/>
@@ -2387,9 +2397,10 @@
       <c r="M7" s="8"/>
       <c r="N7" s="8"/>
       <c r="O7" s="8"/>
-      <c r="P7" s="73"/>
-    </row>
-    <row r="8" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P7" s="8"/>
+      <c r="Q7" s="73"/>
+    </row>
+    <row r="8" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="27"/>
       <c r="C8" s="43"/>
@@ -2405,9 +2416,10 @@
       <c r="M8" s="8"/>
       <c r="N8" s="8"/>
       <c r="O8" s="8"/>
-      <c r="P8" s="73"/>
-    </row>
-    <row r="9" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P8" s="8"/>
+      <c r="Q8" s="73"/>
+    </row>
+    <row r="9" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="30" t="s">
         <v>4</v>
@@ -2440,22 +2452,25 @@
         <v>340</v>
       </c>
       <c r="L9" s="30" t="s">
+        <v>381</v>
+      </c>
+      <c r="M9" s="30" t="s">
         <v>360</v>
       </c>
-      <c r="M9" s="30" t="s">
+      <c r="N9" s="30" t="s">
         <v>361</v>
       </c>
-      <c r="N9" s="30" t="s">
+      <c r="O9" s="30" t="s">
         <v>362</v>
       </c>
-      <c r="O9" s="32" t="s">
+      <c r="P9" s="32" t="s">
         <v>363</v>
       </c>
-      <c r="P9" s="32" t="s">
+      <c r="Q9" s="32" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="10" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="38">
         <f>ROW(B10) - ROW($B$9)</f>
@@ -2489,24 +2504,28 @@
         <v>2</v>
       </c>
       <c r="L10" s="46">
+        <f>K10*5</f>
+        <v>10</v>
+      </c>
+      <c r="M10" s="46">
         <v>11</v>
       </c>
-      <c r="M10" s="53">
+      <c r="N10" s="53">
         <v>0.32690000000000002</v>
       </c>
-      <c r="N10" s="53">
-        <f>M10*L10</f>
+      <c r="O10" s="53">
+        <f t="shared" ref="O10:O41" si="0">N10*M10</f>
         <v>3.5959000000000003</v>
       </c>
-      <c r="O10" s="48"/>
-      <c r="P10" s="49"/>
-      <c r="T10" s="69"/>
-      <c r="X10" s="69"/>
-    </row>
-    <row r="11" spans="1:24" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P10" s="48"/>
+      <c r="Q10" s="49"/>
+      <c r="U10" s="69"/>
+      <c r="Y10" s="69"/>
+    </row>
+    <row r="11" spans="1:25" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="38">
-        <f t="shared" ref="B11:B84" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B84" si="1">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="60" t="s">
@@ -2537,21 +2556,25 @@
         <v>3</v>
       </c>
       <c r="L11" s="50">
+        <f t="shared" ref="L11:L74" si="2">K11*5</f>
+        <v>15</v>
+      </c>
+      <c r="M11" s="50">
         <v>16</v>
       </c>
-      <c r="M11" s="54">
+      <c r="N11" s="54">
         <v>0.48799999999999999</v>
       </c>
-      <c r="N11" s="54">
-        <f>M11*L11</f>
+      <c r="O11" s="54">
+        <f t="shared" si="0"/>
         <v>7.8079999999999998</v>
       </c>
-      <c r="O11" s="52"/>
       <c r="P11" s="52"/>
-      <c r="T11" s="69"/>
-      <c r="X11" s="69"/>
-    </row>
-    <row r="12" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q11" s="52"/>
+      <c r="U11" s="69"/>
+      <c r="Y11" s="69"/>
+    </row>
+    <row r="12" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="38">
         <f>ROW(B12) - ROW($B$9)</f>
@@ -2585,24 +2608,28 @@
         <v>15</v>
       </c>
       <c r="L12" s="46">
+        <f t="shared" si="2"/>
+        <v>75</v>
+      </c>
+      <c r="M12" s="46">
         <v>100</v>
       </c>
-      <c r="M12" s="53">
+      <c r="N12" s="53">
         <v>8.6000000000000007E-2</v>
       </c>
-      <c r="N12" s="53">
-        <f>M12*L12</f>
+      <c r="O12" s="53">
+        <f t="shared" si="0"/>
         <v>8.6000000000000014</v>
       </c>
-      <c r="O12" s="48"/>
-      <c r="P12" s="49"/>
-      <c r="T12" s="69"/>
-      <c r="X12" s="69"/>
-    </row>
-    <row r="13" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P12" s="48"/>
+      <c r="Q12" s="49"/>
+      <c r="U12" s="69"/>
+      <c r="Y12" s="69"/>
+    </row>
+    <row r="13" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="C13" s="60" t="s">
@@ -2633,21 +2660,25 @@
         <v>1</v>
       </c>
       <c r="L13" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M13" s="50">
         <v>6</v>
       </c>
-      <c r="M13" s="54">
+      <c r="N13" s="54">
         <v>0.89249999999999996</v>
       </c>
-      <c r="N13" s="54">
-        <f>M13*L13</f>
+      <c r="O13" s="54">
+        <f t="shared" si="0"/>
         <v>5.3549999999999995</v>
       </c>
-      <c r="O13" s="52"/>
       <c r="P13" s="52"/>
-      <c r="T13" s="69"/>
-      <c r="X13" s="69"/>
-    </row>
-    <row r="14" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q13" s="52"/>
+      <c r="U13" s="69"/>
+      <c r="Y13" s="69"/>
+    </row>
+    <row r="14" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="38">
         <f>ROW(B14) - ROW($B$9)</f>
@@ -2681,24 +2712,28 @@
         <v>4</v>
       </c>
       <c r="L14" s="46">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M14" s="46">
         <v>30</v>
       </c>
-      <c r="M14" s="53">
+      <c r="N14" s="53">
         <v>0.1153</v>
       </c>
-      <c r="N14" s="53">
-        <f>M14*L14</f>
+      <c r="O14" s="53">
+        <f t="shared" si="0"/>
         <v>3.4590000000000001</v>
       </c>
-      <c r="O14" s="48"/>
-      <c r="P14" s="49"/>
-      <c r="T14" s="69"/>
-      <c r="X14" s="69"/>
-    </row>
-    <row r="15" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P14" s="48"/>
+      <c r="Q14" s="49"/>
+      <c r="U14" s="69"/>
+      <c r="Y14" s="69"/>
+    </row>
+    <row r="15" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="C15" s="60" t="s">
@@ -2729,21 +2764,25 @@
         <v>2</v>
       </c>
       <c r="L15" s="50">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M15" s="50">
         <v>100</v>
       </c>
-      <c r="M15" s="54">
+      <c r="N15" s="54">
         <v>8.2799999999999999E-2</v>
       </c>
-      <c r="N15" s="54">
-        <f>M15*L15</f>
+      <c r="O15" s="54">
+        <f t="shared" si="0"/>
         <v>8.2799999999999994</v>
       </c>
-      <c r="O15" s="52"/>
       <c r="P15" s="52"/>
-      <c r="T15" s="69"/>
-      <c r="X15" s="69"/>
-    </row>
-    <row r="16" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q15" s="52"/>
+      <c r="U15" s="69"/>
+      <c r="Y15" s="69"/>
+    </row>
+    <row r="16" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="38">
         <f>ROW(B16) - ROW($B$9)</f>
@@ -2777,24 +2816,28 @@
         <v>10</v>
       </c>
       <c r="L16" s="46">
+        <f t="shared" si="2"/>
+        <v>50</v>
+      </c>
+      <c r="M16" s="46">
         <v>100</v>
       </c>
-      <c r="M16" s="53">
+      <c r="N16" s="53">
         <v>8.4199999999999997E-2</v>
       </c>
-      <c r="N16" s="53">
-        <f>M16*L16</f>
+      <c r="O16" s="53">
+        <f t="shared" si="0"/>
         <v>8.42</v>
       </c>
-      <c r="O16" s="48"/>
-      <c r="P16" s="49"/>
-      <c r="T16" s="69"/>
-      <c r="X16" s="69"/>
-    </row>
-    <row r="17" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P16" s="48"/>
+      <c r="Q16" s="49"/>
+      <c r="U16" s="69"/>
+      <c r="Y16" s="69"/>
+    </row>
+    <row r="17" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="C17" s="60" t="s">
@@ -2825,21 +2868,25 @@
         <v>2</v>
       </c>
       <c r="L17" s="50">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M17" s="50">
         <v>20</v>
       </c>
-      <c r="M17" s="54">
+      <c r="N17" s="54">
         <v>9.4200000000000006E-2</v>
       </c>
-      <c r="N17" s="54">
-        <f>M17*L17</f>
+      <c r="O17" s="54">
+        <f t="shared" si="0"/>
         <v>1.8840000000000001</v>
       </c>
-      <c r="O17" s="52"/>
       <c r="P17" s="52"/>
-      <c r="T17" s="69"/>
-      <c r="X17" s="69"/>
-    </row>
-    <row r="18" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q17" s="52"/>
+      <c r="U17" s="69"/>
+      <c r="Y17" s="69"/>
+    </row>
+    <row r="18" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="38">
         <f>ROW(B18) - ROW($B$9)</f>
@@ -2873,24 +2920,28 @@
         <v>1</v>
       </c>
       <c r="L18" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M18" s="46">
         <v>100</v>
       </c>
-      <c r="M18" s="53">
+      <c r="N18" s="53">
         <v>8.5100000000000009E-2</v>
       </c>
-      <c r="N18" s="53">
-        <f>M18*L18</f>
+      <c r="O18" s="53">
+        <f t="shared" si="0"/>
         <v>8.5100000000000016</v>
       </c>
-      <c r="O18" s="48"/>
-      <c r="P18" s="49"/>
-      <c r="T18" s="69"/>
-      <c r="X18" s="69"/>
-    </row>
-    <row r="19" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P18" s="48"/>
+      <c r="Q18" s="49"/>
+      <c r="U18" s="69"/>
+      <c r="Y18" s="69"/>
+    </row>
+    <row r="19" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="C19" s="60" t="s">
@@ -2921,21 +2972,25 @@
         <v>2</v>
       </c>
       <c r="L19" s="50">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M19" s="50">
         <v>20</v>
       </c>
-      <c r="M19" s="54">
+      <c r="N19" s="54">
         <v>0.1129</v>
       </c>
-      <c r="N19" s="54">
-        <f>M19*L19</f>
+      <c r="O19" s="54">
+        <f t="shared" si="0"/>
         <v>2.258</v>
       </c>
-      <c r="O19" s="52"/>
       <c r="P19" s="52"/>
-      <c r="T19" s="69"/>
-      <c r="X19" s="69"/>
-    </row>
-    <row r="20" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q19" s="52"/>
+      <c r="U19" s="69"/>
+      <c r="Y19" s="69"/>
+    </row>
+    <row r="20" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="38">
         <f>ROW(B20) - ROW($B$9)</f>
@@ -2969,24 +3024,28 @@
         <v>2</v>
       </c>
       <c r="L20" s="46">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M20" s="46">
         <v>100</v>
       </c>
-      <c r="M20" s="53">
+      <c r="N20" s="53">
         <v>8.2900000000000001E-2</v>
       </c>
-      <c r="N20" s="53">
-        <f>M20*L20</f>
+      <c r="O20" s="53">
+        <f t="shared" si="0"/>
         <v>8.2900000000000009</v>
       </c>
-      <c r="O20" s="48"/>
-      <c r="P20" s="49"/>
-      <c r="T20" s="69"/>
-      <c r="X20" s="69"/>
-    </row>
-    <row r="21" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P20" s="48"/>
+      <c r="Q20" s="49"/>
+      <c r="U20" s="69"/>
+      <c r="Y20" s="69"/>
+    </row>
+    <row r="21" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="C21" s="60" t="s">
@@ -3017,21 +3076,25 @@
         <v>1</v>
       </c>
       <c r="L21" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M21" s="50">
         <v>100</v>
       </c>
-      <c r="M21" s="54">
+      <c r="N21" s="54">
         <v>8.3699999999999997E-2</v>
       </c>
-      <c r="N21" s="54">
-        <f>M21*L21</f>
+      <c r="O21" s="54">
+        <f t="shared" si="0"/>
         <v>8.3699999999999992</v>
       </c>
-      <c r="O21" s="52"/>
       <c r="P21" s="52"/>
-      <c r="T21" s="69"/>
-      <c r="X21" s="69"/>
-    </row>
-    <row r="22" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q21" s="52"/>
+      <c r="U21" s="69"/>
+      <c r="Y21" s="69"/>
+    </row>
+    <row r="22" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="38">
         <f>ROW(B22) - ROW($B$9)</f>
@@ -3065,24 +3128,28 @@
         <v>2</v>
       </c>
       <c r="L22" s="46">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M22" s="46">
         <v>20</v>
       </c>
-      <c r="M22" s="53">
+      <c r="N22" s="53">
         <v>0.11210000000000001</v>
       </c>
-      <c r="N22" s="53">
-        <f>M22*L22</f>
+      <c r="O22" s="53">
+        <f t="shared" si="0"/>
         <v>2.242</v>
       </c>
-      <c r="O22" s="48"/>
-      <c r="P22" s="49"/>
-      <c r="T22" s="69"/>
-      <c r="X22" s="69"/>
-    </row>
-    <row r="23" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P22" s="48"/>
+      <c r="Q22" s="49"/>
+      <c r="U22" s="69"/>
+      <c r="Y22" s="69"/>
+    </row>
+    <row r="23" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="C23" s="60" t="s">
@@ -3113,24 +3180,28 @@
         <v>1</v>
       </c>
       <c r="L23" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M23" s="50">
         <v>100</v>
       </c>
-      <c r="M23" s="54">
+      <c r="N23" s="54">
         <v>8.3900000000000002E-2</v>
       </c>
-      <c r="N23" s="54">
-        <f>M23*L23</f>
+      <c r="O23" s="54">
+        <f t="shared" si="0"/>
         <v>8.39</v>
       </c>
-      <c r="O23" s="52"/>
       <c r="P23" s="52"/>
-      <c r="T23" s="69"/>
-      <c r="X23" s="69"/>
-    </row>
-    <row r="24" spans="1:24" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q23" s="52"/>
+      <c r="U23" s="69"/>
+      <c r="Y23" s="69"/>
+    </row>
+    <row r="24" spans="1:25" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="C24" s="59" t="s">
@@ -3161,21 +3232,25 @@
         <v>1</v>
       </c>
       <c r="L24" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M24" s="46">
         <v>10</v>
       </c>
-      <c r="M24" s="53">
+      <c r="N24" s="53">
         <v>0.1797</v>
       </c>
-      <c r="N24" s="53">
-        <f>M24*L24</f>
+      <c r="O24" s="53">
+        <f t="shared" si="0"/>
         <v>1.7969999999999999</v>
       </c>
-      <c r="O24" s="48"/>
-      <c r="P24" s="49"/>
-      <c r="T24" s="69"/>
-      <c r="X24" s="69"/>
-    </row>
-    <row r="25" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P24" s="48"/>
+      <c r="Q24" s="49"/>
+      <c r="U24" s="69"/>
+      <c r="Y24" s="69"/>
+    </row>
+    <row r="25" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="38">
         <f>ROW(B25) - ROW($B$9)</f>
@@ -3209,24 +3284,28 @@
         <v>3</v>
       </c>
       <c r="L25" s="50">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="M25" s="50">
         <v>20</v>
       </c>
-      <c r="M25" s="54">
+      <c r="N25" s="54">
         <v>0.14419999999999999</v>
       </c>
-      <c r="N25" s="54">
-        <f>M25*L25</f>
+      <c r="O25" s="54">
+        <f t="shared" si="0"/>
         <v>2.8839999999999999</v>
       </c>
-      <c r="O25" s="52"/>
       <c r="P25" s="52"/>
-      <c r="T25" s="69"/>
-      <c r="X25" s="69"/>
-    </row>
-    <row r="26" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q25" s="52"/>
+      <c r="U25" s="69"/>
+      <c r="Y25" s="69"/>
+    </row>
+    <row r="26" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="C26" s="59" t="s">
@@ -3257,21 +3336,25 @@
         <v>3</v>
       </c>
       <c r="L26" s="46">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="M26" s="46">
         <v>20</v>
       </c>
-      <c r="M26" s="53">
+      <c r="N26" s="53">
         <v>0.11890000000000001</v>
       </c>
-      <c r="N26" s="53">
-        <f>M26*L26</f>
+      <c r="O26" s="53">
+        <f t="shared" si="0"/>
         <v>2.3780000000000001</v>
       </c>
-      <c r="O26" s="48"/>
-      <c r="P26" s="49"/>
-      <c r="T26" s="69"/>
-      <c r="X26" s="69"/>
-    </row>
-    <row r="27" spans="1:24" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P26" s="48"/>
+      <c r="Q26" s="49"/>
+      <c r="U26" s="69"/>
+      <c r="Y26" s="69"/>
+    </row>
+    <row r="27" spans="1:25" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="38">
         <f>ROW(B27) - ROW($B$9)</f>
@@ -3305,24 +3388,28 @@
         <v>4</v>
       </c>
       <c r="L27" s="50">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M27" s="50">
         <v>50</v>
       </c>
-      <c r="M27" s="54">
+      <c r="N27" s="54">
         <v>8.9700000000000002E-2</v>
       </c>
-      <c r="N27" s="54">
-        <f>M27*L27</f>
+      <c r="O27" s="54">
+        <f t="shared" si="0"/>
         <v>4.4850000000000003</v>
       </c>
-      <c r="O27" s="52"/>
       <c r="P27" s="52"/>
-      <c r="T27" s="69"/>
-      <c r="X27" s="69"/>
-    </row>
-    <row r="28" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q27" s="52"/>
+      <c r="U27" s="69"/>
+      <c r="Y27" s="69"/>
+    </row>
+    <row r="28" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>19</v>
       </c>
       <c r="C28" s="59" t="s">
@@ -3353,21 +3440,25 @@
         <v>1</v>
       </c>
       <c r="L28" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M28" s="46">
         <v>10</v>
       </c>
-      <c r="M28" s="53">
+      <c r="N28" s="53">
         <v>0.13639999999999999</v>
       </c>
-      <c r="N28" s="53">
-        <f>M28*L28</f>
+      <c r="O28" s="53">
+        <f t="shared" si="0"/>
         <v>1.3639999999999999</v>
       </c>
-      <c r="O28" s="48"/>
-      <c r="P28" s="49"/>
-      <c r="T28" s="69"/>
-      <c r="X28" s="69"/>
-    </row>
-    <row r="29" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P28" s="48"/>
+      <c r="Q28" s="49"/>
+      <c r="U28" s="69"/>
+      <c r="Y28" s="69"/>
+    </row>
+    <row r="29" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="38">
         <f>ROW(B29) - ROW($B$9)</f>
@@ -3401,24 +3492,28 @@
         <v>1</v>
       </c>
       <c r="L29" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M29" s="50">
         <v>10</v>
       </c>
-      <c r="M29" s="54">
+      <c r="N29" s="54">
         <v>0.14510000000000001</v>
       </c>
-      <c r="N29" s="54">
-        <f>M29*L29</f>
+      <c r="O29" s="54">
+        <f t="shared" si="0"/>
         <v>1.4510000000000001</v>
       </c>
-      <c r="O29" s="52"/>
       <c r="P29" s="52"/>
-      <c r="T29" s="69"/>
-      <c r="X29" s="69"/>
-    </row>
-    <row r="30" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q29" s="52"/>
+      <c r="U29" s="69"/>
+      <c r="Y29" s="69"/>
+    </row>
+    <row r="30" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>21</v>
       </c>
       <c r="C30" s="59" t="s">
@@ -3449,21 +3544,25 @@
         <v>1</v>
       </c>
       <c r="L30" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M30" s="46">
         <v>20</v>
       </c>
-      <c r="M30" s="53">
+      <c r="N30" s="53">
         <v>0.1055</v>
       </c>
-      <c r="N30" s="53">
-        <f>M30*L30</f>
+      <c r="O30" s="53">
+        <f t="shared" si="0"/>
         <v>2.11</v>
       </c>
-      <c r="O30" s="48"/>
-      <c r="P30" s="49"/>
-      <c r="T30" s="69"/>
-      <c r="X30" s="69"/>
-    </row>
-    <row r="31" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P30" s="48"/>
+      <c r="Q30" s="49"/>
+      <c r="U30" s="69"/>
+      <c r="Y30" s="69"/>
+    </row>
+    <row r="31" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="38">
         <f>ROW(B31) - ROW($B$9)</f>
@@ -3497,24 +3596,28 @@
         <v>1</v>
       </c>
       <c r="L31" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M31" s="50">
         <v>10</v>
       </c>
-      <c r="M31" s="54">
+      <c r="N31" s="54">
         <v>0.20069999999999999</v>
       </c>
-      <c r="N31" s="54">
-        <f>M31*L31</f>
+      <c r="O31" s="54">
+        <f t="shared" si="0"/>
         <v>2.0069999999999997</v>
       </c>
-      <c r="O31" s="52"/>
       <c r="P31" s="52"/>
-      <c r="T31" s="69"/>
-      <c r="X31" s="69"/>
-    </row>
-    <row r="32" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q31" s="52"/>
+      <c r="U31" s="69"/>
+      <c r="Y31" s="69"/>
+    </row>
+    <row r="32" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>23</v>
       </c>
       <c r="C32" s="59" t="s">
@@ -3545,21 +3648,25 @@
         <v>1</v>
       </c>
       <c r="L32" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M32" s="46">
         <v>10</v>
       </c>
-      <c r="M32" s="53">
+      <c r="N32" s="53">
         <v>0.15029999999999999</v>
       </c>
-      <c r="N32" s="53">
-        <f>M32*L32</f>
+      <c r="O32" s="53">
+        <f t="shared" si="0"/>
         <v>1.5029999999999999</v>
       </c>
-      <c r="O32" s="48"/>
-      <c r="P32" s="49"/>
-      <c r="T32" s="69"/>
-      <c r="X32" s="69"/>
-    </row>
-    <row r="33" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P32" s="48"/>
+      <c r="Q32" s="49"/>
+      <c r="U32" s="69"/>
+      <c r="Y32" s="69"/>
+    </row>
+    <row r="33" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="38">
         <f>ROW(B33) - ROW($B$9)</f>
@@ -3593,24 +3700,28 @@
         <v>1</v>
       </c>
       <c r="L33" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M33" s="50">
         <v>10</v>
       </c>
-      <c r="M33" s="54">
+      <c r="N33" s="54">
         <v>0.16839999999999999</v>
       </c>
-      <c r="N33" s="54">
-        <f>M33*L33</f>
+      <c r="O33" s="54">
+        <f t="shared" si="0"/>
         <v>1.6839999999999999</v>
       </c>
-      <c r="O33" s="52"/>
       <c r="P33" s="52"/>
-      <c r="T33" s="69"/>
-      <c r="X33" s="69"/>
-    </row>
-    <row r="34" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q33" s="52"/>
+      <c r="U33" s="69"/>
+      <c r="Y33" s="69"/>
+    </row>
+    <row r="34" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
       <c r="C34" s="59" t="s">
@@ -3641,21 +3752,25 @@
         <v>1</v>
       </c>
       <c r="L34" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M34" s="46">
         <v>10</v>
       </c>
-      <c r="M34" s="53">
+      <c r="N34" s="53">
         <v>0.1409</v>
       </c>
-      <c r="N34" s="53">
-        <f>M34*L34</f>
+      <c r="O34" s="53">
+        <f t="shared" si="0"/>
         <v>1.409</v>
       </c>
-      <c r="O34" s="48"/>
-      <c r="P34" s="49"/>
-      <c r="T34" s="69"/>
-      <c r="X34" s="69"/>
-    </row>
-    <row r="35" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P34" s="48"/>
+      <c r="Q34" s="49"/>
+      <c r="U34" s="69"/>
+      <c r="Y34" s="69"/>
+    </row>
+    <row r="35" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="38">
         <f>ROW(B35) - ROW($B$9)</f>
@@ -3689,24 +3804,28 @@
         <v>1</v>
       </c>
       <c r="L35" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M35" s="50">
         <v>6</v>
       </c>
-      <c r="M35" s="54">
+      <c r="N35" s="54">
         <v>0.83399999999999996</v>
       </c>
-      <c r="N35" s="54">
-        <f>M35*L35</f>
+      <c r="O35" s="54">
+        <f t="shared" si="0"/>
         <v>5.0039999999999996</v>
       </c>
-      <c r="O35" s="52"/>
       <c r="P35" s="52"/>
-      <c r="T35" s="69"/>
-      <c r="X35" s="69"/>
-    </row>
-    <row r="36" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q35" s="52"/>
+      <c r="U35" s="69"/>
+      <c r="Y35" s="69"/>
+    </row>
+    <row r="36" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>27</v>
       </c>
       <c r="C36" s="59" t="s">
@@ -3737,21 +3856,25 @@
         <v>1</v>
       </c>
       <c r="L36" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M36" s="46">
         <v>10</v>
       </c>
-      <c r="M36" s="53">
+      <c r="N36" s="53">
         <v>0.1633</v>
       </c>
-      <c r="N36" s="53">
-        <f>M36*L36</f>
+      <c r="O36" s="53">
+        <f t="shared" si="0"/>
         <v>1.633</v>
       </c>
-      <c r="O36" s="48"/>
-      <c r="P36" s="49"/>
-      <c r="T36" s="69"/>
-      <c r="X36" s="69"/>
-    </row>
-    <row r="37" spans="1:24" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P36" s="48"/>
+      <c r="Q36" s="49"/>
+      <c r="U36" s="69"/>
+      <c r="Y36" s="69"/>
+    </row>
+    <row r="37" spans="1:25" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="38">
         <f>ROW(B37) - ROW($B$9)</f>
@@ -3785,24 +3908,28 @@
         <v>1</v>
       </c>
       <c r="L37" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M37" s="50">
         <v>10</v>
       </c>
-      <c r="M37" s="54">
+      <c r="N37" s="54">
         <v>0.10730000000000001</v>
       </c>
-      <c r="N37" s="54">
-        <f>M37*L37</f>
+      <c r="O37" s="54">
+        <f t="shared" si="0"/>
         <v>1.073</v>
       </c>
-      <c r="O37" s="52"/>
       <c r="P37" s="52"/>
-      <c r="T37" s="69"/>
-      <c r="X37" s="69"/>
-    </row>
-    <row r="38" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q37" s="52"/>
+      <c r="U37" s="69"/>
+      <c r="Y37" s="69"/>
+    </row>
+    <row r="38" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>29</v>
       </c>
       <c r="C38" s="59" t="s">
@@ -3833,21 +3960,25 @@
         <v>8</v>
       </c>
       <c r="L38" s="46">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
+      <c r="M38" s="46">
         <v>50</v>
       </c>
-      <c r="M38" s="53">
+      <c r="N38" s="53">
         <v>9.5899999999999999E-2</v>
       </c>
-      <c r="N38" s="53">
-        <f>M38*L38</f>
+      <c r="O38" s="53">
+        <f t="shared" si="0"/>
         <v>4.7949999999999999</v>
       </c>
-      <c r="O38" s="48"/>
-      <c r="P38" s="49"/>
-      <c r="T38" s="69"/>
-      <c r="X38" s="69"/>
-    </row>
-    <row r="39" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P38" s="48"/>
+      <c r="Q38" s="49"/>
+      <c r="U38" s="69"/>
+      <c r="Y38" s="69"/>
+    </row>
+    <row r="39" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="38">
         <f>ROW(B39) - ROW($B$9)</f>
@@ -3881,24 +4012,28 @@
         <v>1</v>
       </c>
       <c r="L39" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M39" s="50">
         <v>10</v>
       </c>
-      <c r="M39" s="54">
+      <c r="N39" s="54">
         <v>0.1192</v>
       </c>
-      <c r="N39" s="54">
-        <f>M39*L39</f>
+      <c r="O39" s="54">
+        <f t="shared" si="0"/>
         <v>1.1919999999999999</v>
       </c>
-      <c r="O39" s="52"/>
       <c r="P39" s="52"/>
-      <c r="T39" s="69"/>
-      <c r="X39" s="69"/>
-    </row>
-    <row r="40" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q39" s="52"/>
+      <c r="U39" s="69"/>
+      <c r="Y39" s="69"/>
+    </row>
+    <row r="40" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>31</v>
       </c>
       <c r="C40" s="59" t="s">
@@ -3929,21 +4064,25 @@
         <v>1</v>
       </c>
       <c r="L40" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M40" s="46">
         <v>6</v>
       </c>
-      <c r="M40" s="53">
+      <c r="N40" s="53">
         <v>0.56879999999999997</v>
       </c>
-      <c r="N40" s="53">
-        <f>M40*L40</f>
+      <c r="O40" s="53">
+        <f t="shared" si="0"/>
         <v>3.4127999999999998</v>
       </c>
-      <c r="O40" s="48"/>
-      <c r="P40" s="49"/>
-      <c r="T40" s="69"/>
-      <c r="X40" s="69"/>
-    </row>
-    <row r="41" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P40" s="48"/>
+      <c r="Q40" s="49"/>
+      <c r="U40" s="69"/>
+      <c r="Y40" s="69"/>
+    </row>
+    <row r="41" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="38">
         <f>ROW(B41) - ROW($B$9)</f>
@@ -3977,24 +4116,28 @@
         <v>1</v>
       </c>
       <c r="L41" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M41" s="50">
         <v>20</v>
       </c>
-      <c r="M41" s="54">
+      <c r="N41" s="54">
         <v>0.11260000000000001</v>
       </c>
-      <c r="N41" s="54">
-        <f>M41*L41</f>
+      <c r="O41" s="54">
+        <f t="shared" si="0"/>
         <v>2.2520000000000002</v>
       </c>
-      <c r="O41" s="52"/>
       <c r="P41" s="52"/>
-      <c r="T41" s="69"/>
-      <c r="X41" s="69"/>
-    </row>
-    <row r="42" spans="1:24" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q41" s="52"/>
+      <c r="U41" s="69"/>
+      <c r="Y41" s="69"/>
+    </row>
+    <row r="42" spans="1:25" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>33</v>
       </c>
       <c r="C42" s="59" t="s">
@@ -4025,21 +4168,25 @@
         <v>1</v>
       </c>
       <c r="L42" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M42" s="46">
         <v>10</v>
       </c>
-      <c r="M42" s="53">
+      <c r="N42" s="53">
         <v>0.1381</v>
       </c>
-      <c r="N42" s="53">
-        <f>M42*L42</f>
+      <c r="O42" s="53">
+        <f t="shared" ref="O42:O73" si="3">N42*M42</f>
         <v>1.381</v>
       </c>
-      <c r="O42" s="48"/>
-      <c r="P42" s="49"/>
-      <c r="T42" s="69"/>
-      <c r="X42" s="69"/>
-    </row>
-    <row r="43" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P42" s="48"/>
+      <c r="Q42" s="49"/>
+      <c r="U42" s="69"/>
+      <c r="Y42" s="69"/>
+    </row>
+    <row r="43" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="38">
         <f>ROW(B43) - ROW($B$9)</f>
@@ -4073,24 +4220,28 @@
         <v>1</v>
       </c>
       <c r="L43" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M43" s="50">
         <v>20</v>
       </c>
-      <c r="M43" s="54">
+      <c r="N43" s="54">
         <v>0.11549999999999999</v>
       </c>
-      <c r="N43" s="54">
-        <f>M43*L43</f>
+      <c r="O43" s="54">
+        <f t="shared" si="3"/>
         <v>2.3099999999999996</v>
       </c>
-      <c r="O43" s="52"/>
       <c r="P43" s="52"/>
-      <c r="T43" s="69"/>
-      <c r="X43" s="69"/>
-    </row>
-    <row r="44" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q43" s="52"/>
+      <c r="U43" s="69"/>
+      <c r="Y43" s="69"/>
+    </row>
+    <row r="44" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>35</v>
       </c>
       <c r="C44" s="59" t="s">
@@ -4116,20 +4267,24 @@
       <c r="K44" s="47">
         <v>2</v>
       </c>
-      <c r="L44" s="46"/>
-      <c r="M44" s="53">
+      <c r="L44" s="46">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M44" s="46"/>
+      <c r="N44" s="53">
         <v>0.08</v>
       </c>
-      <c r="N44" s="53">
-        <f>M44*L44</f>
+      <c r="O44" s="53">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="O44" s="48"/>
-      <c r="P44" s="49"/>
-      <c r="T44" s="69"/>
-      <c r="X44" s="69"/>
-    </row>
-    <row r="45" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P44" s="48"/>
+      <c r="Q44" s="49"/>
+      <c r="U44" s="69"/>
+      <c r="Y44" s="69"/>
+    </row>
+    <row r="45" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="38">
         <f>ROW(B45) - ROW($B$9)</f>
@@ -4163,24 +4318,28 @@
         <v>6</v>
       </c>
       <c r="L45" s="50">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
+      <c r="M45" s="50">
         <v>40</v>
       </c>
-      <c r="M45" s="54">
+      <c r="N45" s="54">
         <v>0.1096</v>
       </c>
-      <c r="N45" s="54">
-        <f>M45*L45</f>
+      <c r="O45" s="54">
+        <f t="shared" si="3"/>
         <v>4.3840000000000003</v>
       </c>
-      <c r="O45" s="52"/>
       <c r="P45" s="52"/>
-      <c r="T45" s="69"/>
-      <c r="X45" s="69"/>
-    </row>
-    <row r="46" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q45" s="52"/>
+      <c r="U45" s="69"/>
+      <c r="Y45" s="69"/>
+    </row>
+    <row r="46" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>37</v>
       </c>
       <c r="C46" s="59" t="s">
@@ -4211,21 +4370,25 @@
         <v>4</v>
       </c>
       <c r="L46" s="46">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M46" s="46">
         <v>22</v>
       </c>
-      <c r="M46" s="53">
+      <c r="N46" s="53">
         <v>1.4846000000000001</v>
       </c>
-      <c r="N46" s="53">
-        <f>M46*L46</f>
+      <c r="O46" s="53">
+        <f t="shared" si="3"/>
         <v>32.661200000000001</v>
       </c>
-      <c r="O46" s="48"/>
-      <c r="P46" s="49"/>
-      <c r="T46" s="69"/>
-      <c r="X46" s="69"/>
-    </row>
-    <row r="47" spans="1:24" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P46" s="48"/>
+      <c r="Q46" s="49"/>
+      <c r="U46" s="69"/>
+      <c r="Y46" s="69"/>
+    </row>
+    <row r="47" spans="1:25" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="38">
         <f>ROW(B47) - ROW($B$9)</f>
@@ -4259,24 +4422,28 @@
         <v>1</v>
       </c>
       <c r="L47" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M47" s="50">
         <v>6</v>
       </c>
-      <c r="M47" s="54">
+      <c r="N47" s="54">
         <v>0.51549999999999996</v>
       </c>
-      <c r="N47" s="54">
-        <f>M47*L47</f>
+      <c r="O47" s="54">
+        <f t="shared" si="3"/>
         <v>3.093</v>
       </c>
-      <c r="O47" s="52"/>
       <c r="P47" s="52"/>
-      <c r="T47" s="69"/>
-      <c r="X47" s="69"/>
-    </row>
-    <row r="48" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q47" s="52"/>
+      <c r="U47" s="69"/>
+      <c r="Y47" s="69"/>
+    </row>
+    <row r="48" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>39</v>
       </c>
       <c r="C48" s="59" t="s">
@@ -4307,21 +4474,25 @@
         <v>1</v>
       </c>
       <c r="L48" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M48" s="46">
         <v>100</v>
       </c>
-      <c r="M48" s="53">
+      <c r="N48" s="53">
         <v>8.14E-2</v>
       </c>
-      <c r="N48" s="53">
-        <f>M48*L48</f>
+      <c r="O48" s="53">
+        <f t="shared" si="3"/>
         <v>8.14</v>
       </c>
-      <c r="O48" s="48"/>
-      <c r="P48" s="49"/>
-      <c r="T48" s="69"/>
-      <c r="X48" s="69"/>
-    </row>
-    <row r="49" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P48" s="48"/>
+      <c r="Q48" s="49"/>
+      <c r="U48" s="69"/>
+      <c r="Y48" s="69"/>
+    </row>
+    <row r="49" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="38">
         <f>ROW(B49) - ROW($B$9)</f>
@@ -4355,24 +4526,28 @@
         <v>1</v>
       </c>
       <c r="L49" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M49" s="50">
         <v>20</v>
       </c>
-      <c r="M49" s="54">
+      <c r="N49" s="54">
         <v>0.108</v>
       </c>
-      <c r="N49" s="54">
-        <f>M49*L49</f>
+      <c r="O49" s="54">
+        <f t="shared" si="3"/>
         <v>2.16</v>
       </c>
-      <c r="O49" s="52"/>
       <c r="P49" s="52"/>
-      <c r="T49" s="69"/>
-      <c r="X49" s="69"/>
-    </row>
-    <row r="50" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q49" s="52"/>
+      <c r="U49" s="69"/>
+      <c r="Y49" s="69"/>
+    </row>
+    <row r="50" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>41</v>
       </c>
       <c r="C50" s="59" t="s">
@@ -4403,24 +4578,28 @@
         <v>2</v>
       </c>
       <c r="L50" s="46">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M50" s="46">
         <v>20</v>
       </c>
-      <c r="M50" s="53">
+      <c r="N50" s="53">
         <v>0.1106</v>
       </c>
-      <c r="N50" s="53">
-        <f>M50*L50</f>
+      <c r="O50" s="53">
+        <f t="shared" si="3"/>
         <v>2.2120000000000002</v>
       </c>
-      <c r="O50" s="48"/>
-      <c r="P50" s="49"/>
-      <c r="T50" s="69"/>
-      <c r="X50" s="69"/>
-    </row>
-    <row r="51" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P50" s="48"/>
+      <c r="Q50" s="49"/>
+      <c r="U50" s="69"/>
+      <c r="Y50" s="69"/>
+    </row>
+    <row r="51" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
       <c r="B51" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>42</v>
       </c>
       <c r="C51" s="60" t="s">
@@ -4451,21 +4630,25 @@
         <v>1</v>
       </c>
       <c r="L51" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M51" s="50">
         <v>100</v>
       </c>
-      <c r="M51" s="54">
+      <c r="N51" s="54">
         <v>8.1000000000000003E-2</v>
       </c>
-      <c r="N51" s="54">
-        <f>M51*L51</f>
+      <c r="O51" s="54">
+        <f t="shared" si="3"/>
         <v>8.1</v>
       </c>
-      <c r="O51" s="52"/>
       <c r="P51" s="52"/>
-      <c r="T51" s="69"/>
-      <c r="X51" s="69"/>
-    </row>
-    <row r="52" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q51" s="52"/>
+      <c r="U51" s="69"/>
+      <c r="Y51" s="69"/>
+    </row>
+    <row r="52" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
       <c r="B52" s="38">
         <f>ROW(B52) - ROW($B$9)</f>
@@ -4499,24 +4682,28 @@
         <v>7</v>
       </c>
       <c r="L52" s="46">
+        <f t="shared" si="2"/>
+        <v>35</v>
+      </c>
+      <c r="M52" s="46">
         <v>100</v>
       </c>
-      <c r="M52" s="53">
+      <c r="N52" s="53">
         <v>8.1699999999999995E-2</v>
       </c>
-      <c r="N52" s="53">
-        <f>M52*L52</f>
+      <c r="O52" s="53">
+        <f t="shared" si="3"/>
         <v>8.17</v>
       </c>
-      <c r="O52" s="48"/>
-      <c r="P52" s="49"/>
-      <c r="T52" s="69"/>
-      <c r="X52" s="69"/>
-    </row>
-    <row r="53" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P52" s="48"/>
+      <c r="Q52" s="49"/>
+      <c r="U52" s="69"/>
+      <c r="Y52" s="69"/>
+    </row>
+    <row r="53" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
       <c r="B53" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>44</v>
       </c>
       <c r="C53" s="60" t="s">
@@ -4544,20 +4731,24 @@
       <c r="K53" s="51">
         <v>1</v>
       </c>
-      <c r="L53" s="50"/>
-      <c r="M53" s="54">
+      <c r="L53" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M53" s="50"/>
+      <c r="N53" s="54">
         <v>0.08</v>
       </c>
-      <c r="N53" s="54">
-        <f>M53*L53</f>
+      <c r="O53" s="54">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="O53" s="52"/>
       <c r="P53" s="52"/>
-      <c r="T53" s="69"/>
-      <c r="X53" s="69"/>
-    </row>
-    <row r="54" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q53" s="52"/>
+      <c r="U53" s="69"/>
+      <c r="Y53" s="69"/>
+    </row>
+    <row r="54" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
       <c r="B54" s="38">
         <f>ROW(B54) - ROW($B$9)</f>
@@ -4591,24 +4782,28 @@
         <v>1</v>
       </c>
       <c r="L54" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M54" s="46">
         <v>100</v>
       </c>
-      <c r="M54" s="53">
+      <c r="N54" s="53">
         <v>8.1299999999999997E-2</v>
       </c>
-      <c r="N54" s="53">
-        <f>M54*L54</f>
+      <c r="O54" s="53">
+        <f t="shared" si="3"/>
         <v>8.129999999999999</v>
       </c>
-      <c r="O54" s="48"/>
-      <c r="P54" s="49"/>
-      <c r="T54" s="69"/>
-      <c r="X54" s="69"/>
-    </row>
-    <row r="55" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P54" s="48"/>
+      <c r="Q54" s="49"/>
+      <c r="U54" s="69"/>
+      <c r="Y54" s="69"/>
+    </row>
+    <row r="55" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>46</v>
       </c>
       <c r="C55" s="60" t="s">
@@ -4639,21 +4834,25 @@
         <v>1</v>
       </c>
       <c r="L55" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M55" s="50">
         <v>100</v>
       </c>
-      <c r="M55" s="54">
+      <c r="N55" s="54">
         <v>8.1200000000000008E-2</v>
       </c>
-      <c r="N55" s="54">
-        <f>M55*L55</f>
+      <c r="O55" s="54">
+        <f t="shared" si="3"/>
         <v>8.120000000000001</v>
       </c>
-      <c r="O55" s="52"/>
       <c r="P55" s="52"/>
-      <c r="T55" s="69"/>
-      <c r="X55" s="69"/>
-    </row>
-    <row r="56" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q55" s="52"/>
+      <c r="U55" s="69"/>
+      <c r="Y55" s="69"/>
+    </row>
+    <row r="56" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="38">
         <f>ROW(B56) - ROW($B$9)</f>
@@ -4687,24 +4886,28 @@
         <v>1</v>
       </c>
       <c r="L56" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M56" s="46">
         <v>20</v>
       </c>
-      <c r="M56" s="53">
+      <c r="N56" s="53">
         <v>0.11030000000000001</v>
       </c>
-      <c r="N56" s="53">
-        <f>M56*L56</f>
+      <c r="O56" s="53">
+        <f t="shared" si="3"/>
         <v>2.2060000000000004</v>
       </c>
-      <c r="O56" s="48"/>
-      <c r="P56" s="49"/>
-      <c r="T56" s="69"/>
-      <c r="X56" s="69"/>
-    </row>
-    <row r="57" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P56" s="48"/>
+      <c r="Q56" s="49"/>
+      <c r="U56" s="69"/>
+      <c r="Y56" s="69"/>
+    </row>
+    <row r="57" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>48</v>
       </c>
       <c r="C57" s="60" t="s">
@@ -4735,21 +4938,25 @@
         <v>8</v>
       </c>
       <c r="L57" s="50">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
+      <c r="M57" s="50">
         <v>100</v>
       </c>
-      <c r="M57" s="54">
+      <c r="N57" s="54">
         <v>8.1200000000000008E-2</v>
       </c>
-      <c r="N57" s="54">
-        <f>M57*L57</f>
+      <c r="O57" s="54">
+        <f t="shared" si="3"/>
         <v>8.120000000000001</v>
       </c>
-      <c r="O57" s="52"/>
       <c r="P57" s="52"/>
-      <c r="T57" s="69"/>
-      <c r="X57" s="69"/>
-    </row>
-    <row r="58" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q57" s="52"/>
+      <c r="U57" s="69"/>
+      <c r="Y57" s="69"/>
+    </row>
+    <row r="58" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
       <c r="B58" s="38">
         <f>ROW(B58) - ROW($B$9)</f>
@@ -4783,24 +4990,28 @@
         <v>1</v>
       </c>
       <c r="L58" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M58" s="46">
         <v>10</v>
       </c>
-      <c r="M58" s="53">
+      <c r="N58" s="53">
         <v>0.16389999999999999</v>
       </c>
-      <c r="N58" s="53">
-        <f>M58*L58</f>
+      <c r="O58" s="53">
+        <f t="shared" si="3"/>
         <v>1.6389999999999998</v>
       </c>
-      <c r="O58" s="48"/>
-      <c r="P58" s="49"/>
-      <c r="T58" s="69"/>
-      <c r="X58" s="69"/>
-    </row>
-    <row r="59" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P58" s="48"/>
+      <c r="Q58" s="49"/>
+      <c r="U58" s="69"/>
+      <c r="Y58" s="69"/>
+    </row>
+    <row r="59" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
       <c r="B59" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>50</v>
       </c>
       <c r="C59" s="60" t="s">
@@ -4831,21 +5042,25 @@
         <v>3</v>
       </c>
       <c r="L59" s="50">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="M59" s="50">
         <v>100</v>
       </c>
-      <c r="M59" s="54">
+      <c r="N59" s="54">
         <v>8.1299999999999997E-2</v>
       </c>
-      <c r="N59" s="54">
-        <f>M59*L59</f>
+      <c r="O59" s="54">
+        <f t="shared" si="3"/>
         <v>8.129999999999999</v>
       </c>
-      <c r="O59" s="52"/>
       <c r="P59" s="52"/>
-      <c r="T59" s="69"/>
-      <c r="X59" s="69"/>
-    </row>
-    <row r="60" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q59" s="52"/>
+      <c r="U59" s="69"/>
+      <c r="Y59" s="69"/>
+    </row>
+    <row r="60" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
       <c r="B60" s="38">
         <f>ROW(B60) - ROW($B$9)</f>
@@ -4879,24 +5094,28 @@
         <v>1</v>
       </c>
       <c r="L60" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M60" s="46">
         <v>10</v>
       </c>
-      <c r="M60" s="53">
+      <c r="N60" s="53">
         <v>0.14400000000000002</v>
       </c>
-      <c r="N60" s="53">
-        <f>M60*L60</f>
+      <c r="O60" s="53">
+        <f t="shared" si="3"/>
         <v>1.4400000000000002</v>
       </c>
-      <c r="O60" s="48"/>
-      <c r="P60" s="49"/>
-      <c r="T60" s="69"/>
-      <c r="X60" s="69"/>
-    </row>
-    <row r="61" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P60" s="48"/>
+      <c r="Q60" s="49"/>
+      <c r="U60" s="69"/>
+      <c r="Y60" s="69"/>
+    </row>
+    <row r="61" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
       <c r="B61" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>52</v>
       </c>
       <c r="C61" s="60" t="s">
@@ -4927,21 +5146,25 @@
         <v>4</v>
       </c>
       <c r="L61" s="50">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M61" s="50">
         <v>100</v>
       </c>
-      <c r="M61" s="54">
+      <c r="N61" s="54">
         <v>8.1299999999999997E-2</v>
       </c>
-      <c r="N61" s="54">
-        <f>M61*L61</f>
+      <c r="O61" s="54">
+        <f t="shared" si="3"/>
         <v>8.129999999999999</v>
       </c>
-      <c r="O61" s="52"/>
       <c r="P61" s="52"/>
-      <c r="T61" s="69"/>
-      <c r="X61" s="69"/>
-    </row>
-    <row r="62" spans="1:24" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q61" s="52"/>
+      <c r="U61" s="69"/>
+      <c r="Y61" s="69"/>
+    </row>
+    <row r="62" spans="1:25" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
       <c r="B62" s="38">
         <f>ROW(B62) - ROW($B$9)</f>
@@ -4975,21 +5198,25 @@
         <v>1</v>
       </c>
       <c r="L62" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M62" s="46">
         <v>20</v>
       </c>
-      <c r="M62" s="53">
+      <c r="N62" s="53">
         <v>0.10150000000000001</v>
       </c>
-      <c r="N62" s="53">
-        <f>M62*L62</f>
+      <c r="O62" s="53">
+        <f t="shared" si="3"/>
         <v>2.0300000000000002</v>
       </c>
-      <c r="O62" s="48"/>
-      <c r="P62" s="49"/>
-      <c r="T62" s="69"/>
-      <c r="X62" s="69"/>
-    </row>
-    <row r="63" spans="1:24" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P62" s="48"/>
+      <c r="Q62" s="49"/>
+      <c r="U62" s="69"/>
+      <c r="Y62" s="69"/>
+    </row>
+    <row r="63" spans="1:25" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
       <c r="B63" s="38">
         <f>ROW(B63) - ROW($B$9)</f>
@@ -5023,24 +5250,28 @@
         <v>1</v>
       </c>
       <c r="L63" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M63" s="50">
         <v>50</v>
       </c>
-      <c r="M63" s="54">
+      <c r="N63" s="54">
         <v>8.4100000000000008E-2</v>
       </c>
-      <c r="N63" s="54">
-        <f>M63*L63</f>
+      <c r="O63" s="54">
+        <f t="shared" si="3"/>
         <v>4.2050000000000001</v>
       </c>
-      <c r="O63" s="52"/>
       <c r="P63" s="52"/>
-      <c r="T63" s="69"/>
-      <c r="X63" s="69"/>
-    </row>
-    <row r="64" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q63" s="52"/>
+      <c r="U63" s="69"/>
+      <c r="Y63" s="69"/>
+    </row>
+    <row r="64" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
       <c r="B64" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>55</v>
       </c>
       <c r="C64" s="59" t="s">
@@ -5071,21 +5302,25 @@
         <v>1</v>
       </c>
       <c r="L64" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M64" s="46">
         <v>100</v>
       </c>
-      <c r="M64" s="53">
+      <c r="N64" s="53">
         <v>8.1900000000000001E-2</v>
       </c>
-      <c r="N64" s="53">
-        <f>M64*L64</f>
+      <c r="O64" s="53">
+        <f t="shared" si="3"/>
         <v>8.19</v>
       </c>
-      <c r="O64" s="48"/>
-      <c r="P64" s="49"/>
-      <c r="T64" s="69"/>
-      <c r="X64" s="69"/>
-    </row>
-    <row r="65" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P64" s="48"/>
+      <c r="Q64" s="49"/>
+      <c r="U64" s="69"/>
+      <c r="Y64" s="69"/>
+    </row>
+    <row r="65" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1"/>
       <c r="B65" s="38">
         <f>ROW(B65) - ROW($B$9)</f>
@@ -5119,24 +5354,28 @@
         <v>2</v>
       </c>
       <c r="L65" s="50">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M65" s="50">
         <v>100</v>
       </c>
-      <c r="M65" s="54">
+      <c r="N65" s="54">
         <v>8.1299999999999997E-2</v>
       </c>
-      <c r="N65" s="54">
-        <f>M65*L65</f>
+      <c r="O65" s="54">
+        <f t="shared" si="3"/>
         <v>8.129999999999999</v>
       </c>
-      <c r="O65" s="52"/>
       <c r="P65" s="52"/>
-      <c r="T65" s="69"/>
-      <c r="X65" s="69"/>
-    </row>
-    <row r="66" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q65" s="52"/>
+      <c r="U65" s="69"/>
+      <c r="Y65" s="69"/>
+    </row>
+    <row r="66" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1"/>
       <c r="B66" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>57</v>
       </c>
       <c r="C66" s="59" t="s">
@@ -5167,21 +5406,25 @@
         <v>1</v>
       </c>
       <c r="L66" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M66" s="46">
         <v>20</v>
       </c>
-      <c r="M66" s="53">
+      <c r="N66" s="53">
         <v>0.1182</v>
       </c>
-      <c r="N66" s="53">
-        <f>M66*L66</f>
+      <c r="O66" s="53">
+        <f t="shared" si="3"/>
         <v>2.3639999999999999</v>
       </c>
-      <c r="O66" s="48"/>
-      <c r="P66" s="49"/>
-      <c r="T66" s="69"/>
-      <c r="X66" s="69"/>
-    </row>
-    <row r="67" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P66" s="48"/>
+      <c r="Q66" s="49"/>
+      <c r="U66" s="69"/>
+      <c r="Y66" s="69"/>
+    </row>
+    <row r="67" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
       <c r="B67" s="38">
         <f>ROW(B67) - ROW($B$9)</f>
@@ -5215,24 +5458,28 @@
         <v>1</v>
       </c>
       <c r="L67" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M67" s="50">
         <v>100</v>
       </c>
-      <c r="M67" s="54">
+      <c r="N67" s="54">
         <v>8.14E-2</v>
       </c>
-      <c r="N67" s="54">
-        <f>M67*L67</f>
+      <c r="O67" s="54">
+        <f t="shared" si="3"/>
         <v>8.14</v>
       </c>
-      <c r="O67" s="52"/>
       <c r="P67" s="52"/>
-      <c r="T67" s="69"/>
-      <c r="X67" s="69"/>
-    </row>
-    <row r="68" spans="1:24" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q67" s="52"/>
+      <c r="U67" s="69"/>
+      <c r="Y67" s="69"/>
+    </row>
+    <row r="68" spans="1:25" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
       <c r="B68" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>59</v>
       </c>
       <c r="C68" s="59" t="s">
@@ -5263,21 +5510,25 @@
         <v>1</v>
       </c>
       <c r="L68" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M68" s="46">
         <v>10</v>
       </c>
-      <c r="M68" s="53">
+      <c r="N68" s="53">
         <v>0.22870000000000001</v>
       </c>
-      <c r="N68" s="53">
-        <f>M68*L68</f>
+      <c r="O68" s="53">
+        <f t="shared" si="3"/>
         <v>2.2869999999999999</v>
       </c>
-      <c r="O68" s="48"/>
-      <c r="P68" s="49"/>
-      <c r="T68" s="69"/>
-      <c r="X68" s="69"/>
-    </row>
-    <row r="69" spans="1:24" ht="84.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P68" s="48"/>
+      <c r="Q68" s="49"/>
+      <c r="U68" s="69"/>
+      <c r="Y68" s="69"/>
+    </row>
+    <row r="69" spans="1:25" ht="84.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
       <c r="B69" s="38">
         <f>ROW(B69) - ROW($B$9)</f>
@@ -5310,24 +5561,28 @@
       <c r="K69" s="51">
         <v>38</v>
       </c>
-      <c r="L69" s="50" t="s">
-        <v>356</v>
-      </c>
-      <c r="M69" s="54" t="s">
+      <c r="L69" s="50">
+        <f t="shared" si="2"/>
+        <v>190</v>
+      </c>
+      <c r="M69" s="50" t="s">
         <v>356</v>
       </c>
       <c r="N69" s="54" t="s">
         <v>356</v>
       </c>
-      <c r="O69" s="52"/>
+      <c r="O69" s="54" t="s">
+        <v>356</v>
+      </c>
       <c r="P69" s="52"/>
-      <c r="T69" s="69"/>
-      <c r="X69" s="69"/>
-    </row>
-    <row r="70" spans="1:24" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q69" s="52"/>
+      <c r="U69" s="69"/>
+      <c r="Y69" s="69"/>
+    </row>
+    <row r="70" spans="1:25" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1"/>
       <c r="B70" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>61</v>
       </c>
       <c r="C70" s="59" t="s">
@@ -5358,21 +5613,25 @@
         <v>2</v>
       </c>
       <c r="L70" s="46">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M70" s="46">
         <v>20</v>
       </c>
-      <c r="M70" s="53">
+      <c r="N70" s="53">
         <v>0.14300000000000002</v>
       </c>
-      <c r="N70" s="53">
-        <f>M70*L70</f>
+      <c r="O70" s="53">
+        <f t="shared" ref="O70:O84" si="4">N70*M70</f>
         <v>2.8600000000000003</v>
       </c>
-      <c r="O70" s="48"/>
-      <c r="P70" s="49"/>
-      <c r="T70" s="69"/>
-      <c r="X70" s="69"/>
-    </row>
-    <row r="71" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P70" s="48"/>
+      <c r="Q70" s="49"/>
+      <c r="U70" s="69"/>
+      <c r="Y70" s="69"/>
+    </row>
+    <row r="71" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="1"/>
       <c r="B71" s="38">
         <f>ROW(B71) - ROW($B$9)</f>
@@ -5406,24 +5665,28 @@
         <v>1</v>
       </c>
       <c r="L71" s="50">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M71" s="50">
         <v>6</v>
       </c>
-      <c r="M71" s="54">
+      <c r="N71" s="54">
         <v>0.5706</v>
       </c>
-      <c r="N71" s="54">
-        <f>M71*L71</f>
+      <c r="O71" s="54">
+        <f t="shared" si="4"/>
         <v>3.4236</v>
       </c>
-      <c r="O71" s="52"/>
       <c r="P71" s="52"/>
-      <c r="T71" s="69"/>
-      <c r="X71" s="69"/>
-    </row>
-    <row r="72" spans="1:24" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q71" s="52"/>
+      <c r="U71" s="69"/>
+      <c r="Y71" s="69"/>
+    </row>
+    <row r="72" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1"/>
       <c r="B72" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>63</v>
       </c>
       <c r="C72" s="59" t="s">
@@ -5444,29 +5707,35 @@
       <c r="H72" s="46" t="s">
         <v>290</v>
       </c>
-      <c r="I72" s="46"/>
+      <c r="I72" s="46" t="s">
+        <v>356</v>
+      </c>
       <c r="J72" s="46" t="s">
         <v>356</v>
       </c>
       <c r="K72" s="47">
         <v>1</v>
       </c>
-      <c r="L72" s="46"/>
-      <c r="M72" s="53">
-        <v>0.08</v>
+      <c r="L72" s="80">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M72" s="46">
+        <v>6</v>
       </c>
       <c r="N72" s="53">
-        <f>M72*L72</f>
-        <v>0</v>
-      </c>
-      <c r="O72" s="68" t="s">
-        <v>379</v>
-      </c>
-      <c r="P72" s="49"/>
-      <c r="T72" s="69"/>
-      <c r="X72" s="69"/>
-    </row>
-    <row r="73" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>10.95</v>
+      </c>
+      <c r="O72" s="53">
+        <f t="shared" si="4"/>
+        <v>65.699999999999989</v>
+      </c>
+      <c r="P72" s="68"/>
+      <c r="Q72" s="49"/>
+      <c r="U72" s="69"/>
+      <c r="Y72" s="69"/>
+    </row>
+    <row r="73" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
       <c r="B73" s="38">
         <f>ROW(B73) - ROW($B$9)</f>
@@ -5500,24 +5769,28 @@
         <v>2</v>
       </c>
       <c r="L73" s="50">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M73" s="50">
         <v>11</v>
       </c>
-      <c r="M73" s="54">
+      <c r="N73" s="54">
         <v>0.87529999999999997</v>
       </c>
-      <c r="N73" s="54">
-        <f>M73*L73</f>
+      <c r="O73" s="54">
+        <f t="shared" si="4"/>
         <v>9.6282999999999994</v>
       </c>
-      <c r="O73" s="52"/>
       <c r="P73" s="52"/>
-      <c r="T73" s="69"/>
-      <c r="X73" s="69"/>
-    </row>
-    <row r="74" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q73" s="52"/>
+      <c r="U73" s="69"/>
+      <c r="Y73" s="69"/>
+    </row>
+    <row r="74" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
       <c r="B74" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>65</v>
       </c>
       <c r="C74" s="59" t="s">
@@ -5548,21 +5821,25 @@
         <v>1</v>
       </c>
       <c r="L74" s="46">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M74" s="46">
         <v>6</v>
       </c>
-      <c r="M74" s="53">
+      <c r="N74" s="53">
         <v>0.46390000000000003</v>
       </c>
-      <c r="N74" s="53">
-        <f>M74*L74</f>
+      <c r="O74" s="53">
+        <f t="shared" si="4"/>
         <v>2.7834000000000003</v>
       </c>
-      <c r="O74" s="48"/>
-      <c r="P74" s="49"/>
-      <c r="T74" s="69"/>
-      <c r="X74" s="69"/>
-    </row>
-    <row r="75" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P74" s="48"/>
+      <c r="Q74" s="49"/>
+      <c r="U74" s="69"/>
+      <c r="Y74" s="69"/>
+    </row>
+    <row r="75" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
       <c r="B75" s="38">
         <f>ROW(B75) - ROW($B$9)</f>
@@ -5596,24 +5873,28 @@
         <v>1</v>
       </c>
       <c r="L75" s="50">
+        <f t="shared" ref="L75:L87" si="5">K75*5</f>
+        <v>5</v>
+      </c>
+      <c r="M75" s="50">
         <v>6</v>
       </c>
-      <c r="M75" s="54">
+      <c r="N75" s="54">
         <v>2.6465000000000001</v>
       </c>
-      <c r="N75" s="54">
-        <f>M75*L75</f>
+      <c r="O75" s="54">
+        <f t="shared" si="4"/>
         <v>15.879000000000001</v>
       </c>
-      <c r="O75" s="52"/>
       <c r="P75" s="52"/>
-      <c r="T75" s="69"/>
-      <c r="X75" s="69"/>
-    </row>
-    <row r="76" spans="1:24" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q75" s="52"/>
+      <c r="U75" s="69"/>
+      <c r="Y75" s="69"/>
+    </row>
+    <row r="76" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1"/>
       <c r="B76" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>67</v>
       </c>
       <c r="C76" s="59" t="s">
@@ -5634,29 +5915,35 @@
       <c r="H76" s="46" t="s">
         <v>292</v>
       </c>
-      <c r="I76" s="46"/>
+      <c r="I76" s="46" t="s">
+        <v>356</v>
+      </c>
       <c r="J76" s="46" t="s">
         <v>356</v>
       </c>
       <c r="K76" s="47">
         <v>1</v>
       </c>
-      <c r="L76" s="46"/>
-      <c r="M76" s="53">
-        <v>0.08</v>
+      <c r="L76" s="46">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="M76" s="46">
+        <v>6</v>
       </c>
       <c r="N76" s="53">
-        <f>M76*L76</f>
-        <v>0</v>
-      </c>
-      <c r="O76" s="68" t="s">
-        <v>379</v>
-      </c>
-      <c r="P76" s="49"/>
-      <c r="T76" s="69"/>
-      <c r="X76" s="69"/>
-    </row>
-    <row r="77" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>43.58</v>
+      </c>
+      <c r="O76" s="53">
+        <f t="shared" si="4"/>
+        <v>261.48</v>
+      </c>
+      <c r="P76" s="68"/>
+      <c r="Q76" s="49"/>
+      <c r="U76" s="69"/>
+      <c r="Y76" s="69"/>
+    </row>
+    <row r="77" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1"/>
       <c r="B77" s="38">
         <f>ROW(B77) - ROW($B$9)</f>
@@ -5690,24 +5977,28 @@
         <v>1</v>
       </c>
       <c r="L77" s="50">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="M77" s="50">
         <v>6</v>
       </c>
-      <c r="M77" s="54">
+      <c r="N77" s="54">
         <v>0.8425999999999999</v>
       </c>
-      <c r="N77" s="54">
-        <f>M77*L77</f>
+      <c r="O77" s="54">
+        <f t="shared" si="4"/>
         <v>5.0555999999999992</v>
       </c>
-      <c r="O77" s="52"/>
       <c r="P77" s="52"/>
-      <c r="T77" s="69"/>
-      <c r="X77" s="69"/>
-    </row>
-    <row r="78" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q77" s="52"/>
+      <c r="U77" s="69"/>
+      <c r="Y77" s="69"/>
+    </row>
+    <row r="78" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1"/>
       <c r="B78" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>69</v>
       </c>
       <c r="C78" s="59" t="s">
@@ -5738,21 +6029,25 @@
         <v>1</v>
       </c>
       <c r="L78" s="46">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="M78" s="46">
         <v>6</v>
       </c>
-      <c r="M78" s="53">
+      <c r="N78" s="53">
         <v>4.2904</v>
       </c>
-      <c r="N78" s="53">
-        <f>M78*L78</f>
+      <c r="O78" s="53">
+        <f t="shared" si="4"/>
         <v>25.7424</v>
       </c>
-      <c r="O78" s="48"/>
-      <c r="P78" s="49"/>
-      <c r="T78" s="69"/>
-      <c r="X78" s="69"/>
-    </row>
-    <row r="79" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P78" s="48"/>
+      <c r="Q78" s="49"/>
+      <c r="U78" s="69"/>
+      <c r="Y78" s="69"/>
+    </row>
+    <row r="79" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1"/>
       <c r="B79" s="38">
         <f>ROW(B79) - ROW($B$9)</f>
@@ -5786,24 +6081,28 @@
         <v>1</v>
       </c>
       <c r="L79" s="50">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="M79" s="50">
         <v>6</v>
       </c>
-      <c r="M79" s="54">
+      <c r="N79" s="54">
         <v>1.5626</v>
       </c>
-      <c r="N79" s="54">
-        <f>M79*L79</f>
+      <c r="O79" s="54">
+        <f t="shared" si="4"/>
         <v>9.3756000000000004</v>
       </c>
-      <c r="O79" s="52"/>
       <c r="P79" s="52"/>
-      <c r="T79" s="69"/>
-      <c r="X79" s="69"/>
-    </row>
-    <row r="80" spans="1:24" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q79" s="52"/>
+      <c r="U79" s="69"/>
+      <c r="Y79" s="69"/>
+    </row>
+    <row r="80" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1"/>
       <c r="B80" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>71</v>
       </c>
       <c r="C80" s="59" t="s">
@@ -5821,30 +6120,38 @@
       <c r="G80" s="47" t="s">
         <v>249</v>
       </c>
-      <c r="H80" s="46"/>
-      <c r="I80" s="46"/>
+      <c r="H80" s="46" t="s">
+        <v>356</v>
+      </c>
+      <c r="I80" s="46" t="s">
+        <v>356</v>
+      </c>
       <c r="J80" s="46" t="s">
         <v>356</v>
       </c>
       <c r="K80" s="47">
         <v>1</v>
       </c>
-      <c r="L80" s="46"/>
-      <c r="M80" s="53">
-        <v>0.08</v>
+      <c r="L80" s="46">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="M80" s="46">
+        <v>6</v>
       </c>
       <c r="N80" s="53">
-        <f>M80*L80</f>
-        <v>0</v>
-      </c>
-      <c r="O80" s="68" t="s">
-        <v>379</v>
-      </c>
-      <c r="P80" s="49"/>
-      <c r="T80" s="69"/>
-      <c r="X80" s="69"/>
-    </row>
-    <row r="81" spans="1:24" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>3.28</v>
+      </c>
+      <c r="O80" s="53">
+        <f t="shared" si="4"/>
+        <v>19.68</v>
+      </c>
+      <c r="P80" s="68"/>
+      <c r="Q80" s="49"/>
+      <c r="U80" s="69"/>
+      <c r="Y80" s="69"/>
+    </row>
+    <row r="81" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1"/>
       <c r="B81" s="38">
         <f>ROW(B81) - ROW($B$9)</f>
@@ -5878,24 +6185,28 @@
         <v>1</v>
       </c>
       <c r="L81" s="50">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="M81" s="50">
         <v>6</v>
       </c>
-      <c r="M81" s="54">
+      <c r="N81" s="54">
         <v>0.57230000000000003</v>
       </c>
-      <c r="N81" s="54">
-        <f>M81*L81</f>
+      <c r="O81" s="54">
+        <f t="shared" si="4"/>
         <v>3.4338000000000002</v>
       </c>
-      <c r="O81" s="52"/>
       <c r="P81" s="52"/>
-      <c r="T81" s="69"/>
-      <c r="X81" s="69"/>
-    </row>
-    <row r="82" spans="1:24" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q81" s="52"/>
+      <c r="U81" s="69"/>
+      <c r="Y81" s="69"/>
+    </row>
+    <row r="82" spans="1:25" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1"/>
       <c r="B82" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>73</v>
       </c>
       <c r="C82" s="59" t="s">
@@ -5916,29 +6227,35 @@
       <c r="H82" s="46" t="s">
         <v>297</v>
       </c>
-      <c r="I82" s="46"/>
+      <c r="I82" s="46" t="s">
+        <v>356</v>
+      </c>
       <c r="J82" s="46" t="s">
         <v>356</v>
       </c>
       <c r="K82" s="47">
         <v>1</v>
       </c>
-      <c r="L82" s="46"/>
-      <c r="M82" s="53">
-        <v>0.08</v>
+      <c r="L82" s="46">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="M82" s="46">
+        <v>6</v>
       </c>
       <c r="N82" s="53">
-        <f>M82*L82</f>
-        <v>0</v>
-      </c>
-      <c r="O82" s="68" t="s">
-        <v>379</v>
-      </c>
-      <c r="P82" s="49"/>
-      <c r="T82" s="69"/>
-      <c r="X82" s="69"/>
-    </row>
-    <row r="83" spans="1:24" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1.53</v>
+      </c>
+      <c r="O82" s="53">
+        <f t="shared" si="4"/>
+        <v>9.18</v>
+      </c>
+      <c r="P82" s="68"/>
+      <c r="Q82" s="49"/>
+      <c r="U82" s="69"/>
+      <c r="Y82" s="69"/>
+    </row>
+    <row r="83" spans="1:25" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="1"/>
       <c r="B83" s="38">
         <f>ROW(B83) - ROW($B$9)</f>
@@ -5972,24 +6289,28 @@
         <v>1</v>
       </c>
       <c r="L83" s="50">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="M83" s="50">
         <v>10</v>
       </c>
-      <c r="M83" s="54">
+      <c r="N83" s="54">
         <v>0.16689999999999999</v>
       </c>
-      <c r="N83" s="54">
-        <f>M83*L83</f>
+      <c r="O83" s="54">
+        <f t="shared" si="4"/>
         <v>1.669</v>
       </c>
-      <c r="O83" s="52"/>
       <c r="P83" s="52"/>
-      <c r="T83" s="69"/>
-      <c r="X83" s="69"/>
-    </row>
-    <row r="84" spans="1:24" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q83" s="52"/>
+      <c r="U83" s="69"/>
+      <c r="Y83" s="69"/>
+    </row>
+    <row r="84" spans="1:25" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="1"/>
       <c r="B84" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>75</v>
       </c>
       <c r="C84" s="59" t="s">
@@ -6020,21 +6341,25 @@
         <v>1</v>
       </c>
       <c r="L84" s="46">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="M84" s="46">
         <v>10</v>
       </c>
-      <c r="M84" s="53">
+      <c r="N84" s="53">
         <v>0.192</v>
       </c>
-      <c r="N84" s="53">
-        <f>M84*L84</f>
+      <c r="O84" s="53">
+        <f t="shared" si="4"/>
         <v>1.92</v>
       </c>
-      <c r="O84" s="48"/>
-      <c r="P84" s="49"/>
-      <c r="T84" s="69"/>
-      <c r="X84" s="69"/>
-    </row>
-    <row r="85" spans="1:24" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P84" s="48"/>
+      <c r="Q84" s="49"/>
+      <c r="U84" s="69"/>
+      <c r="Y84" s="69"/>
+    </row>
+    <row r="85" spans="1:25" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="1"/>
       <c r="B85" s="33"/>
       <c r="C85" s="44"/>
@@ -6046,18 +6371,19 @@
       <c r="I85" s="37"/>
       <c r="J85" s="37"/>
       <c r="K85" s="37"/>
-      <c r="L85" s="78" t="s">
+      <c r="L85" s="37"/>
+      <c r="M85" s="78" t="s">
         <v>377</v>
       </c>
-      <c r="M85" s="79"/>
-      <c r="N85" s="66">
-        <f>SUM(N10:N84)</f>
-        <v>363.53860000000009</v>
-      </c>
-      <c r="O85" s="74"/>
-      <c r="P85" s="75"/>
-    </row>
-    <row r="86" spans="1:24" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N85" s="79"/>
+      <c r="O85" s="66">
+        <f>SUM(O10:O84)</f>
+        <v>719.57859999999982</v>
+      </c>
+      <c r="P85" s="74"/>
+      <c r="Q85" s="75"/>
+    </row>
+    <row r="86" spans="1:25" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="1"/>
       <c r="B86" s="25"/>
       <c r="C86" s="45"/>
@@ -6069,28 +6395,29 @@
       <c r="I86" s="10"/>
       <c r="J86" s="10"/>
       <c r="K86" s="10"/>
-      <c r="L86" s="78" t="s">
+      <c r="L86" s="10"/>
+      <c r="M86" s="78" t="s">
         <v>378</v>
       </c>
-      <c r="M86" s="79"/>
-      <c r="N86" s="67">
-        <f>N85/5</f>
-        <v>72.707720000000023</v>
-      </c>
-      <c r="O86" s="76"/>
-      <c r="P86" s="77"/>
-      <c r="X86" s="69"/>
-    </row>
-    <row r="88" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="M88" s="69"/>
+      <c r="N86" s="79"/>
+      <c r="O86" s="67">
+        <f>O85/5</f>
+        <v>143.91571999999996</v>
+      </c>
+      <c r="P86" s="76"/>
+      <c r="Q86" s="77"/>
+      <c r="Y86" s="69"/>
+    </row>
+    <row r="88" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="N88" s="69"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="J1:P1"/>
-    <mergeCell ref="P3:P8"/>
-    <mergeCell ref="O85:P86"/>
-    <mergeCell ref="L85:M85"/>
-    <mergeCell ref="L86:M86"/>
+    <mergeCell ref="J1:Q1"/>
+    <mergeCell ref="Q3:Q8"/>
+    <mergeCell ref="P85:Q86"/>
+    <mergeCell ref="M85:N85"/>
+    <mergeCell ref="M86:N86"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>